<commit_message>
Scrape Selectel Configurable Pre-Build (PCL*) line via calculator API
Формула цены разгадана из фронтового чанка selectel
(seidoPrecustomServersStore): цена = сумма price.rub × count по
компонентам calculator/items (enable, не is_hidden); компонент,
отсутствующий в items, ПРОПУСКАЕТСЯ из цены, но обнуляет наличие —
такие конфиги сайт не показывает (фильтр available_count > 0).
Загадка 12.08 «38 300 ≠ 44 640» решена: id=73 (плата) исчез из items,
PCL67 сейчас скрыт и на сайте.

- _scrape_selectel_precustom: precustom+items через tls_client,
  сборка через общий _selectel_cfg_to_row; GPU-конфиги пропускаются
  (эталоны без GPU); 34 из 113 конфигов доступны = витрина сайта
- canonical_cpu: варианты без «(8x3.6 GHz HT)»-хвоста и с
  восстановленным «Xeon» («Intel Silver 4214R» selectel) — лечит
  и молча не матчившийся PBL57-SSD
- Живой прогон: selectel 190 офферов, +2 матча (MIR-053 PCL33-NVMe,
  MIR-192 PCL07-NVMe); 178 тестов passed
</commit_message>
<xml_diff>
--- a/data/reports/dedicated_competitors_20260817.xlsx
+++ b/data/reports/dedicated_competitors_20260817.xlsx
@@ -2930,7 +2930,7 @@
         <v>100</v>
       </c>
       <c r="M47" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N47" t="n">
         <v>2</v>
@@ -3372,10 +3372,10 @@
         <v>100</v>
       </c>
       <c r="M54" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr"/>
@@ -10630,13 +10630,33 @@
       <c r="G193" t="n">
         <v>59780</v>
       </c>
-      <c r="H193" t="inlineStr"/>
-      <c r="I193" t="inlineStr"/>
-      <c r="J193" t="inlineStr"/>
-      <c r="K193" t="inlineStr"/>
-      <c r="L193" t="inlineStr"/>
-      <c r="M193" t="inlineStr"/>
-      <c r="N193" t="inlineStr"/>
+      <c r="H193" t="n">
+        <v>121240</v>
+      </c>
+      <c r="I193" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="J193" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>PCL07-NVMe</t>
+        </is>
+      </c>
+      <c r="L193" t="n">
+        <v>100</v>
+      </c>
+      <c r="M193" t="n">
+        <v>4</v>
+      </c>
+      <c r="N193" t="n">
+        <v>1</v>
+      </c>
       <c r="O193" t="inlineStr"/>
       <c r="P193" t="inlineStr"/>
       <c r="Q193" t="inlineStr"/>

</xml_diff>